<commit_message>
added more mock data
</commit_message>
<xml_diff>
--- a/mockdata/Binary_Information.xlsx
+++ b/mockdata/Binary_Information.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taylorlaurensergel/Desktop/Honours 26'/IMY/Project/IMY772Project/mockdata/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4342B89B-29E0-D44F-B4E7-C943A037E758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="198">
   <si>
     <t>Sample ID</t>
   </si>
@@ -104,41 +113,537 @@
   </si>
   <si>
     <t>eae, bfpA</t>
+  </si>
+  <si>
+    <t>SAMP-004</t>
+  </si>
+  <si>
+    <t>ISO-104</t>
+  </si>
+  <si>
+    <t>TSp4H</t>
+  </si>
+  <si>
+    <t>Acinetobacter baumannii</t>
+  </si>
+  <si>
+    <t>River water downstream</t>
+  </si>
+  <si>
+    <t>B9</t>
+  </si>
+  <si>
+    <t>SAMP-005</t>
+  </si>
+  <si>
+    <t>ISO-105</t>
+  </si>
+  <si>
+    <t>Pi5</t>
+  </si>
+  <si>
+    <t>B35</t>
+  </si>
+  <si>
+    <t>SAMP-006</t>
+  </si>
+  <si>
+    <t>ISO-106</t>
+  </si>
+  <si>
+    <t>Agr6</t>
+  </si>
+  <si>
+    <t>Pseudomonas aeruginosa</t>
+  </si>
+  <si>
+    <t>River water upstream</t>
+  </si>
+  <si>
+    <t>B14</t>
+  </si>
+  <si>
+    <t>iucC, sitA</t>
+  </si>
+  <si>
+    <t>SAMP-007</t>
+  </si>
+  <si>
+    <t>ISO-107</t>
+  </si>
+  <si>
+    <t>Str7</t>
+  </si>
+  <si>
+    <t>B30</t>
+  </si>
+  <si>
+    <t>SAMP-008</t>
+  </si>
+  <si>
+    <t>ISO-108</t>
+  </si>
+  <si>
+    <t>Agr8</t>
+  </si>
+  <si>
+    <t>Effluent discharge point</t>
+  </si>
+  <si>
+    <t>B6</t>
+  </si>
+  <si>
+    <t>stx1, stx2</t>
+  </si>
+  <si>
+    <t>SAMP-009</t>
+  </si>
+  <si>
+    <t>ISO-109</t>
+  </si>
+  <si>
+    <t>Pi9</t>
+  </si>
+  <si>
+    <t>B5</t>
+  </si>
+  <si>
+    <t>hlyA, fyuA</t>
+  </si>
+  <si>
+    <t>SAMP-010</t>
+  </si>
+  <si>
+    <t>ISO-110</t>
+  </si>
+  <si>
+    <t>Agr10H</t>
+  </si>
+  <si>
+    <t>Treated wastewater output</t>
+  </si>
+  <si>
+    <t>B4</t>
+  </si>
+  <si>
+    <t>SAMP-011</t>
+  </si>
+  <si>
+    <t>ISO-111</t>
+  </si>
+  <si>
+    <t>Pi11H</t>
+  </si>
+  <si>
+    <t>Enterococcus faecalis</t>
+  </si>
+  <si>
+    <t>B32</t>
+  </si>
+  <si>
+    <t>SAMP-012</t>
+  </si>
+  <si>
+    <t>ISO-112</t>
+  </si>
+  <si>
+    <t>Agr12H</t>
+  </si>
+  <si>
+    <t>Hospital drain effluent</t>
+  </si>
+  <si>
+    <t>B38</t>
+  </si>
+  <si>
+    <t>SAMP-013</t>
+  </si>
+  <si>
+    <t>ISO-113</t>
+  </si>
+  <si>
+    <t>Str13</t>
+  </si>
+  <si>
+    <t>B11</t>
+  </si>
+  <si>
+    <t>SAMP-014</t>
+  </si>
+  <si>
+    <t>ISO-114</t>
+  </si>
+  <si>
+    <t>Hos14H</t>
+  </si>
+  <si>
+    <t>csgA, fimH</t>
+  </si>
+  <si>
+    <t>SAMP-015</t>
+  </si>
+  <si>
+    <t>ISO-115</t>
+  </si>
+  <si>
+    <t>Riv15</t>
+  </si>
+  <si>
+    <t>B33</t>
+  </si>
+  <si>
+    <t>SAMP-016</t>
+  </si>
+  <si>
+    <t>ISO-116</t>
+  </si>
+  <si>
+    <t>Hos16H</t>
+  </si>
+  <si>
+    <t>Proteus mirabilis</t>
+  </si>
+  <si>
+    <t>B39</t>
+  </si>
+  <si>
+    <t>SAMP-017</t>
+  </si>
+  <si>
+    <t>ISO-117</t>
+  </si>
+  <si>
+    <t>Pi17</t>
+  </si>
+  <si>
+    <t>SAMP-018</t>
+  </si>
+  <si>
+    <t>ISO-118</t>
+  </si>
+  <si>
+    <t>Hos18H</t>
+  </si>
+  <si>
+    <t>Staphylococcus aureus</t>
+  </si>
+  <si>
+    <t>SAMP-019</t>
+  </si>
+  <si>
+    <t>ISO-119</t>
+  </si>
+  <si>
+    <t>TSp19</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>SAMP-020</t>
+  </si>
+  <si>
+    <t>ISO-120</t>
+  </si>
+  <si>
+    <t>TSp20H</t>
+  </si>
+  <si>
+    <t>SAMP-021</t>
+  </si>
+  <si>
+    <t>ISO-121</t>
+  </si>
+  <si>
+    <t>Pi21H</t>
+  </si>
+  <si>
+    <t>B7</t>
+  </si>
+  <si>
+    <t>SAMP-022</t>
+  </si>
+  <si>
+    <t>ISO-122</t>
+  </si>
+  <si>
+    <t>Eff4</t>
+  </si>
+  <si>
+    <t>B20</t>
+  </si>
+  <si>
+    <t>SAMP-023</t>
+  </si>
+  <si>
+    <t>ISO-123</t>
+  </si>
+  <si>
+    <t>TSp5H</t>
+  </si>
+  <si>
+    <t>papG, hlyD</t>
+  </si>
+  <si>
+    <t>SAMP-024</t>
+  </si>
+  <si>
+    <t>ISO-124</t>
+  </si>
+  <si>
+    <t>Riv6H</t>
+  </si>
+  <si>
+    <t>B36</t>
+  </si>
+  <si>
+    <t>SAMP-025</t>
+  </si>
+  <si>
+    <t>ISO-125</t>
+  </si>
+  <si>
+    <t>Hos7</t>
+  </si>
+  <si>
+    <t>B22</t>
+  </si>
+  <si>
+    <t>SAMP-026</t>
+  </si>
+  <si>
+    <t>ISO-126</t>
+  </si>
+  <si>
+    <t>Riv8H</t>
+  </si>
+  <si>
+    <t>SAMP-027</t>
+  </si>
+  <si>
+    <t>ISO-127</t>
+  </si>
+  <si>
+    <t>TSp9</t>
+  </si>
+  <si>
+    <t>B24</t>
+  </si>
+  <si>
+    <t>SAMP-028</t>
+  </si>
+  <si>
+    <t>ISO-128</t>
+  </si>
+  <si>
+    <t>TSp10H</t>
+  </si>
+  <si>
+    <t>SAMP-029</t>
+  </si>
+  <si>
+    <t>ISO-129</t>
+  </si>
+  <si>
+    <t>Riv11</t>
+  </si>
+  <si>
+    <t>B16</t>
+  </si>
+  <si>
+    <t>SAMP-030</t>
+  </si>
+  <si>
+    <t>ISO-130</t>
+  </si>
+  <si>
+    <t>Pi12</t>
+  </si>
+  <si>
+    <t>Salmonella enterica</t>
+  </si>
+  <si>
+    <t>SAMP-031</t>
+  </si>
+  <si>
+    <t>ISO-131</t>
+  </si>
+  <si>
+    <t>Eff13H</t>
+  </si>
+  <si>
+    <t>SAMP-032</t>
+  </si>
+  <si>
+    <t>ISO-132</t>
+  </si>
+  <si>
+    <t>SAMP-033</t>
+  </si>
+  <si>
+    <t>ISO-133</t>
+  </si>
+  <si>
+    <t>Hos15</t>
+  </si>
+  <si>
+    <t>SAMP-034</t>
+  </si>
+  <si>
+    <t>ISO-134</t>
+  </si>
+  <si>
+    <t>TSp16H</t>
+  </si>
+  <si>
+    <t>SAMP-035</t>
+  </si>
+  <si>
+    <t>ISO-135</t>
+  </si>
+  <si>
+    <t>Riv17H</t>
+  </si>
+  <si>
+    <t>SAMP-036</t>
+  </si>
+  <si>
+    <t>ISO-136</t>
+  </si>
+  <si>
+    <t>Riv18</t>
+  </si>
+  <si>
+    <t>Agricultural runoff</t>
+  </si>
+  <si>
+    <t>SAMP-037</t>
+  </si>
+  <si>
+    <t>ISO-137</t>
+  </si>
+  <si>
+    <t>Pi19H</t>
+  </si>
+  <si>
+    <t>B3</t>
+  </si>
+  <si>
+    <t>SAMP-038</t>
+  </si>
+  <si>
+    <t>ISO-138</t>
+  </si>
+  <si>
+    <t>Riv20</t>
+  </si>
+  <si>
+    <t>SAMP-039</t>
+  </si>
+  <si>
+    <t>ISO-139</t>
+  </si>
+  <si>
+    <t>Hos21</t>
+  </si>
+  <si>
+    <t>SAMP-040</t>
+  </si>
+  <si>
+    <t>ISO-140</t>
+  </si>
+  <si>
+    <t>Riv22</t>
+  </si>
+  <si>
+    <t>B34</t>
+  </si>
+  <si>
+    <t>SAMP-041</t>
+  </si>
+  <si>
+    <t>ISO-141</t>
+  </si>
+  <si>
+    <t>Pi23</t>
+  </si>
+  <si>
+    <t>SAMP-042</t>
+  </si>
+  <si>
+    <t>ISO-142</t>
+  </si>
+  <si>
+    <t>Riv24</t>
+  </si>
+  <si>
+    <t>SAMP-043</t>
+  </si>
+  <si>
+    <t>ISO-143</t>
+  </si>
+  <si>
+    <t>Riv25</t>
+  </si>
+  <si>
+    <t>B25</t>
+  </si>
+  <si>
+    <t>SAMP-044</t>
+  </si>
+  <si>
+    <t>ISO-144</t>
+  </si>
+  <si>
+    <t>Riv26</t>
+  </si>
+  <si>
+    <t>SAMP-045</t>
+  </si>
+  <si>
+    <t>ISO-145</t>
+  </si>
+  <si>
+    <t>Riv27</t>
+  </si>
+  <si>
+    <t>SAMP-046</t>
+  </si>
+  <si>
+    <t>ISO-146</t>
+  </si>
+  <si>
+    <t>Eff28H</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b val="1"/>
+      <b/>
       <sz val="12"/>
       <color indexed="9"/>
       <name val="Helvetica"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color indexed="9"/>
       <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -180,37 +685,43 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -220,25 +731,85 @@
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ff1f1f1f"/>
-      <rgbColor rgb="ffefefef"/>
-      <rgbColor rgb="ffa5a5a5"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FF1F1F1F"/>
+      <rgbColor rgb="FFEFEFEF"/>
+      <rgbColor rgb="FFA5A5A5"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Blank">
   <a:themeElements>
     <a:clrScheme name="Blank">
       <a:dk1>
@@ -440,7 +1011,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -458,7 +1029,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -487,7 +1058,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -512,7 +1083,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -537,7 +1108,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -562,7 +1133,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -587,7 +1158,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -612,7 +1183,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -637,7 +1208,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -662,7 +1233,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -687,7 +1258,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -700,9 +1271,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -719,7 +1296,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -737,7 +1314,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -762,7 +1339,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -787,7 +1364,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -812,7 +1389,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -837,7 +1414,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -862,7 +1439,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -887,7 +1464,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -912,7 +1489,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -937,7 +1514,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -962,7 +1539,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -975,9 +1552,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -991,7 +1574,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1009,7 +1592,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1038,7 +1621,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1063,7 +1646,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1088,7 +1671,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1113,7 +1696,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1138,7 +1721,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1163,7 +1746,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1188,7 +1771,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1213,7 +1796,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1238,7 +1821,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1251,86 +1834,93 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O22"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="13.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O47"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="60.25" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="15" width="16.3516" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="16.3516" style="1" customWidth="1"/>
+    <col min="1" max="16" width="16.33203125" style="1" customWidth="1"/>
+    <col min="17" max="16384" width="16.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="60.55" customHeight="1">
-      <c r="A1" t="s" s="2">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s" s="2">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s" s="2">
+    <row r="1" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="2">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="2">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="2">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s" s="2">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s" s="2">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s" s="2">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s" s="2">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s" s="2">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s" s="2">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="3"/>
       <c r="N1" s="3"/>
       <c r="O1" s="3"/>
     </row>
-    <row r="2" ht="74.55" customHeight="1">
-      <c r="A2" t="s" s="4">
+    <row r="2" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s" s="4">
+      <c r="B2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s" s="4">
+      <c r="C2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s" s="4">
+      <c r="D2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s" s="4">
+      <c r="E2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F2" t="s" s="4">
+      <c r="F2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="s" s="4">
+      <c r="G2" s="4" t="s">
         <v>18</v>
       </c>
       <c r="H2" s="5">
@@ -1352,23 +1942,23 @@
       <c r="N2" s="6"/>
       <c r="O2" s="6"/>
     </row>
-    <row r="3" ht="46.35" customHeight="1">
-      <c r="A3" t="s" s="4">
+    <row r="3" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B3" t="s" s="4">
+      <c r="B3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C3" t="s" s="4">
+      <c r="C3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D3" t="s" s="4">
+      <c r="D3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E3" t="s" s="4">
+      <c r="E3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F3" t="s" s="4">
+      <c r="F3" s="4" t="s">
         <v>24</v>
       </c>
       <c r="G3" s="7"/>
@@ -1391,26 +1981,26 @@
       <c r="N3" s="6"/>
       <c r="O3" s="6"/>
     </row>
-    <row r="4" ht="60.35" customHeight="1">
-      <c r="A4" t="s" s="4">
+    <row r="4" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s" s="4">
+      <c r="B4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s" s="4">
+      <c r="C4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s" s="4">
+      <c r="D4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s" s="4">
+      <c r="E4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F4" t="s" s="4">
+      <c r="F4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G4" t="s" s="4">
+      <c r="G4" s="4" t="s">
         <v>30</v>
       </c>
       <c r="H4" s="5">
@@ -1432,315 +2022,1689 @@
       <c r="N4" s="6"/>
       <c r="O4" s="6"/>
     </row>
-    <row r="5" ht="46.35" customHeight="1">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
+    <row r="5" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="9">
+        <v>0</v>
+      </c>
+      <c r="I5" s="9">
+        <v>1</v>
+      </c>
+      <c r="J5" s="9">
+        <v>0</v>
+      </c>
+      <c r="K5" s="9">
+        <v>0</v>
+      </c>
+      <c r="L5" s="9">
+        <v>0</v>
+      </c>
       <c r="M5" s="8"/>
       <c r="N5" s="8"/>
       <c r="O5" s="8"/>
     </row>
-    <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
+    <row r="6" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9">
+        <v>0</v>
+      </c>
+      <c r="I6" s="9">
+        <v>1</v>
+      </c>
+      <c r="J6" s="9">
+        <v>1</v>
+      </c>
+      <c r="K6" s="9">
+        <v>0</v>
+      </c>
+      <c r="L6" s="9">
+        <v>0</v>
+      </c>
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
       <c r="O6" s="8"/>
     </row>
-    <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
+    <row r="7" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="9">
+        <v>0</v>
+      </c>
+      <c r="I7" s="9">
+        <v>0</v>
+      </c>
+      <c r="J7" s="9">
+        <v>1</v>
+      </c>
+      <c r="K7" s="9">
+        <v>0</v>
+      </c>
+      <c r="L7" s="9">
+        <v>1</v>
+      </c>
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
     </row>
-    <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
+    <row r="8" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="9">
+        <v>1</v>
+      </c>
+      <c r="I8" s="9">
+        <v>0</v>
+      </c>
+      <c r="J8" s="9">
+        <v>1</v>
+      </c>
+      <c r="K8" s="9">
+        <v>1</v>
+      </c>
+      <c r="L8" s="9">
+        <v>0</v>
+      </c>
       <c r="M8" s="8"/>
       <c r="N8" s="8"/>
       <c r="O8" s="8"/>
     </row>
-    <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
+    <row r="9" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="H9" s="9">
+        <v>0</v>
+      </c>
+      <c r="I9" s="9">
+        <v>1</v>
+      </c>
+      <c r="J9" s="9">
+        <v>1</v>
+      </c>
+      <c r="K9" s="9">
+        <v>1</v>
+      </c>
+      <c r="L9" s="9">
+        <v>1</v>
+      </c>
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
     </row>
-    <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
+    <row r="10" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" s="9">
+        <v>0</v>
+      </c>
+      <c r="I10" s="9">
+        <v>0</v>
+      </c>
+      <c r="J10" s="9">
+        <v>1</v>
+      </c>
+      <c r="K10" s="9">
+        <v>1</v>
+      </c>
+      <c r="L10" s="9">
+        <v>1</v>
+      </c>
       <c r="M10" s="8"/>
       <c r="N10" s="8"/>
       <c r="O10" s="8"/>
     </row>
-    <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
-      <c r="L11" s="8"/>
+    <row r="11" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="H11" s="9">
+        <v>0</v>
+      </c>
+      <c r="I11" s="9">
+        <v>1</v>
+      </c>
+      <c r="J11" s="9">
+        <v>1</v>
+      </c>
+      <c r="K11" s="9">
+        <v>1</v>
+      </c>
+      <c r="L11" s="9">
+        <v>0</v>
+      </c>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
       <c r="O11" s="8"/>
     </row>
-    <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
+    <row r="12" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9">
+        <v>1</v>
+      </c>
+      <c r="I12" s="9">
+        <v>0</v>
+      </c>
+      <c r="J12" s="9">
+        <v>1</v>
+      </c>
+      <c r="K12" s="9">
+        <v>0</v>
+      </c>
+      <c r="L12" s="9">
+        <v>0</v>
+      </c>
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
       <c r="O12" s="8"/>
     </row>
-    <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
+    <row r="13" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9">
+        <v>1</v>
+      </c>
+      <c r="I13" s="9">
+        <v>0</v>
+      </c>
+      <c r="J13" s="9">
+        <v>0</v>
+      </c>
+      <c r="K13" s="9">
+        <v>1</v>
+      </c>
+      <c r="L13" s="9">
+        <v>0</v>
+      </c>
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
       <c r="O13" s="8"/>
     </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="8"/>
+    <row r="14" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9">
+        <v>0</v>
+      </c>
+      <c r="I14" s="9">
+        <v>1</v>
+      </c>
+      <c r="J14" s="9">
+        <v>1</v>
+      </c>
+      <c r="K14" s="9">
+        <v>1</v>
+      </c>
+      <c r="L14" s="9">
+        <v>1</v>
+      </c>
       <c r="M14" s="8"/>
       <c r="N14" s="8"/>
       <c r="O14" s="8"/>
     </row>
-    <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
+    <row r="15" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="H15" s="9">
+        <v>1</v>
+      </c>
+      <c r="I15" s="9">
+        <v>0</v>
+      </c>
+      <c r="J15" s="9">
+        <v>1</v>
+      </c>
+      <c r="K15" s="9">
+        <v>1</v>
+      </c>
+      <c r="L15" s="9">
+        <v>0</v>
+      </c>
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
       <c r="O15" s="8"/>
     </row>
-    <row r="16" ht="20.05" customHeight="1">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
+    <row r="16" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="H16" s="9">
+        <v>1</v>
+      </c>
+      <c r="I16" s="9">
+        <v>0</v>
+      </c>
+      <c r="J16" s="9">
+        <v>0</v>
+      </c>
+      <c r="K16" s="9">
+        <v>1</v>
+      </c>
+      <c r="L16" s="9">
+        <v>0</v>
+      </c>
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
       <c r="O16" s="8"/>
     </row>
-    <row r="17" ht="20.05" customHeight="1">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
+    <row r="17" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H17" s="9">
+        <v>1</v>
+      </c>
+      <c r="I17" s="9">
+        <v>0</v>
+      </c>
+      <c r="J17" s="9">
+        <v>0</v>
+      </c>
+      <c r="K17" s="9">
+        <v>1</v>
+      </c>
+      <c r="L17" s="9">
+        <v>1</v>
+      </c>
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
       <c r="O17" s="8"/>
     </row>
-    <row r="18" ht="20.05" customHeight="1">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
+    <row r="18" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A18" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="H18" s="9">
+        <v>0</v>
+      </c>
+      <c r="I18" s="9">
+        <v>0</v>
+      </c>
+      <c r="J18" s="9">
+        <v>1</v>
+      </c>
+      <c r="K18" s="9">
+        <v>0</v>
+      </c>
+      <c r="L18" s="9">
+        <v>1</v>
+      </c>
       <c r="M18" s="8"/>
       <c r="N18" s="8"/>
       <c r="O18" s="8"/>
     </row>
-    <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
+    <row r="19" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="H19" s="9">
+        <v>1</v>
+      </c>
+      <c r="I19" s="9">
+        <v>1</v>
+      </c>
+      <c r="J19" s="9">
+        <v>1</v>
+      </c>
+      <c r="K19" s="9">
+        <v>1</v>
+      </c>
+      <c r="L19" s="9">
+        <v>1</v>
+      </c>
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
       <c r="O19" s="8"/>
     </row>
-    <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
+    <row r="20" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="H20" s="9">
+        <v>0</v>
+      </c>
+      <c r="I20" s="9">
+        <v>0</v>
+      </c>
+      <c r="J20" s="9">
+        <v>0</v>
+      </c>
+      <c r="K20" s="9">
+        <v>0</v>
+      </c>
+      <c r="L20" s="9">
+        <v>0</v>
+      </c>
       <c r="M20" s="8"/>
       <c r="N20" s="8"/>
       <c r="O20" s="8"/>
     </row>
-    <row r="21" ht="20.05" customHeight="1">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
+    <row r="21" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="H21" s="9">
+        <v>1</v>
+      </c>
+      <c r="I21" s="9">
+        <v>1</v>
+      </c>
+      <c r="J21" s="9">
+        <v>0</v>
+      </c>
+      <c r="K21" s="9">
+        <v>0</v>
+      </c>
+      <c r="L21" s="9">
+        <v>1</v>
+      </c>
       <c r="M21" s="8"/>
       <c r="N21" s="8"/>
       <c r="O21" s="8"/>
     </row>
-    <row r="22" ht="20.05" customHeight="1">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="8"/>
+    <row r="22" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="H22" s="9">
+        <v>1</v>
+      </c>
+      <c r="I22" s="9">
+        <v>1</v>
+      </c>
+      <c r="J22" s="9">
+        <v>1</v>
+      </c>
+      <c r="K22" s="9">
+        <v>1</v>
+      </c>
+      <c r="L22" s="9">
+        <v>1</v>
+      </c>
       <c r="M22" s="8"/>
       <c r="N22" s="8"/>
       <c r="O22" s="8"/>
     </row>
+    <row r="23" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="H23" s="10">
+        <v>1</v>
+      </c>
+      <c r="I23" s="10">
+        <v>0</v>
+      </c>
+      <c r="J23" s="10">
+        <v>0</v>
+      </c>
+      <c r="K23" s="10">
+        <v>1</v>
+      </c>
+      <c r="L23" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G24" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="H24" s="10">
+        <v>0</v>
+      </c>
+      <c r="I24" s="10">
+        <v>0</v>
+      </c>
+      <c r="J24" s="10">
+        <v>1</v>
+      </c>
+      <c r="K24" s="10">
+        <v>1</v>
+      </c>
+      <c r="L24" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="H25" s="10">
+        <v>0</v>
+      </c>
+      <c r="I25" s="10">
+        <v>0</v>
+      </c>
+      <c r="J25" s="10">
+        <v>1</v>
+      </c>
+      <c r="K25" s="10">
+        <v>0</v>
+      </c>
+      <c r="L25" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="G26" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H26" s="10">
+        <v>1</v>
+      </c>
+      <c r="I26" s="10">
+        <v>1</v>
+      </c>
+      <c r="J26" s="10">
+        <v>1</v>
+      </c>
+      <c r="K26" s="10">
+        <v>0</v>
+      </c>
+      <c r="L26" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A27" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="G27" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H27" s="10">
+        <v>1</v>
+      </c>
+      <c r="I27" s="10">
+        <v>0</v>
+      </c>
+      <c r="J27" s="10">
+        <v>1</v>
+      </c>
+      <c r="K27" s="10">
+        <v>1</v>
+      </c>
+      <c r="L27" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H28" s="10">
+        <v>1</v>
+      </c>
+      <c r="I28" s="10">
+        <v>0</v>
+      </c>
+      <c r="J28" s="10">
+        <v>0</v>
+      </c>
+      <c r="K28" s="10">
+        <v>1</v>
+      </c>
+      <c r="L28" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A29" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="H29" s="10">
+        <v>1</v>
+      </c>
+      <c r="I29" s="10">
+        <v>0</v>
+      </c>
+      <c r="J29" s="10">
+        <v>0</v>
+      </c>
+      <c r="K29" s="10">
+        <v>0</v>
+      </c>
+      <c r="L29" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A30" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="H30" s="10">
+        <v>0</v>
+      </c>
+      <c r="I30" s="10">
+        <v>0</v>
+      </c>
+      <c r="J30" s="10">
+        <v>1</v>
+      </c>
+      <c r="K30" s="10">
+        <v>0</v>
+      </c>
+      <c r="L30" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H31" s="10">
+        <v>0</v>
+      </c>
+      <c r="I31" s="10">
+        <v>0</v>
+      </c>
+      <c r="J31" s="10">
+        <v>0</v>
+      </c>
+      <c r="K31" s="10">
+        <v>1</v>
+      </c>
+      <c r="L31" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A32" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="H32" s="10">
+        <v>1</v>
+      </c>
+      <c r="I32" s="10">
+        <v>0</v>
+      </c>
+      <c r="J32" s="10">
+        <v>0</v>
+      </c>
+      <c r="K32" s="10">
+        <v>1</v>
+      </c>
+      <c r="L32" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A33" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="H33" s="10">
+        <v>1</v>
+      </c>
+      <c r="I33" s="10">
+        <v>1</v>
+      </c>
+      <c r="J33" s="10">
+        <v>1</v>
+      </c>
+      <c r="K33" s="10">
+        <v>0</v>
+      </c>
+      <c r="L33" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A34" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G34" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H34" s="10">
+        <v>1</v>
+      </c>
+      <c r="I34" s="10">
+        <v>1</v>
+      </c>
+      <c r="J34" s="10">
+        <v>0</v>
+      </c>
+      <c r="K34" s="10">
+        <v>1</v>
+      </c>
+      <c r="L34" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F35" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G35" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="H35" s="10">
+        <v>1</v>
+      </c>
+      <c r="I35" s="10">
+        <v>1</v>
+      </c>
+      <c r="J35" s="10">
+        <v>0</v>
+      </c>
+      <c r="K35" s="10">
+        <v>0</v>
+      </c>
+      <c r="L35" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A36" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F36" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="H36" s="10">
+        <v>1</v>
+      </c>
+      <c r="I36" s="10">
+        <v>1</v>
+      </c>
+      <c r="J36" s="10">
+        <v>0</v>
+      </c>
+      <c r="K36" s="10">
+        <v>1</v>
+      </c>
+      <c r="L36" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A37" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="H37" s="10">
+        <v>1</v>
+      </c>
+      <c r="I37" s="10">
+        <v>1</v>
+      </c>
+      <c r="J37" s="10">
+        <v>0</v>
+      </c>
+      <c r="K37" s="10">
+        <v>0</v>
+      </c>
+      <c r="L37" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A38" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H38" s="10">
+        <v>1</v>
+      </c>
+      <c r="I38" s="10">
+        <v>0</v>
+      </c>
+      <c r="J38" s="10">
+        <v>1</v>
+      </c>
+      <c r="K38" s="10">
+        <v>1</v>
+      </c>
+      <c r="L38" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A39" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="H39" s="10">
+        <v>1</v>
+      </c>
+      <c r="I39" s="10">
+        <v>0</v>
+      </c>
+      <c r="J39" s="10">
+        <v>0</v>
+      </c>
+      <c r="K39" s="10">
+        <v>1</v>
+      </c>
+      <c r="L39" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A40" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="B40" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G40" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="H40" s="10">
+        <v>1</v>
+      </c>
+      <c r="I40" s="10">
+        <v>1</v>
+      </c>
+      <c r="J40" s="10">
+        <v>1</v>
+      </c>
+      <c r="K40" s="10">
+        <v>1</v>
+      </c>
+      <c r="L40" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A41" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="H41" s="10">
+        <v>0</v>
+      </c>
+      <c r="I41" s="10">
+        <v>1</v>
+      </c>
+      <c r="J41" s="10">
+        <v>1</v>
+      </c>
+      <c r="K41" s="10">
+        <v>0</v>
+      </c>
+      <c r="L41" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A42" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F42" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G42" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H42" s="10">
+        <v>0</v>
+      </c>
+      <c r="I42" s="10">
+        <v>1</v>
+      </c>
+      <c r="J42" s="10">
+        <v>0</v>
+      </c>
+      <c r="K42" s="10">
+        <v>0</v>
+      </c>
+      <c r="L42" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A43" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="F43" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="H43" s="10">
+        <v>0</v>
+      </c>
+      <c r="I43" s="10">
+        <v>1</v>
+      </c>
+      <c r="J43" s="10">
+        <v>1</v>
+      </c>
+      <c r="K43" s="10">
+        <v>0</v>
+      </c>
+      <c r="L43" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A44" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B44" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E44" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F44" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="G44" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="H44" s="10">
+        <v>0</v>
+      </c>
+      <c r="I44" s="10">
+        <v>1</v>
+      </c>
+      <c r="J44" s="10">
+        <v>0</v>
+      </c>
+      <c r="K44" s="10">
+        <v>1</v>
+      </c>
+      <c r="L44" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A45" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="B45" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F45" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G45" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="H45" s="10">
+        <v>0</v>
+      </c>
+      <c r="I45" s="10">
+        <v>0</v>
+      </c>
+      <c r="J45" s="10">
+        <v>1</v>
+      </c>
+      <c r="K45" s="10">
+        <v>0</v>
+      </c>
+      <c r="L45" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A46" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="B46" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="E46" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G46" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="H46" s="10">
+        <v>1</v>
+      </c>
+      <c r="I46" s="10">
+        <v>1</v>
+      </c>
+      <c r="J46" s="10">
+        <v>0</v>
+      </c>
+      <c r="K46" s="10">
+        <v>1</v>
+      </c>
+      <c r="L46" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" ht="60.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A47" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B47" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G47" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="H47" s="10">
+        <v>0</v>
+      </c>
+      <c r="I47" s="10">
+        <v>1</v>
+      </c>
+      <c r="J47" s="10">
+        <v>0</v>
+      </c>
+      <c r="K47" s="10">
+        <v>0</v>
+      </c>
+      <c r="L47" s="10">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.27777800000000002" footer="0.27777800000000002"/>
+  <pageSetup scale="72" orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>